<commit_message>
114th Commit: Epic Seven Updated
</commit_message>
<xml_diff>
--- a/EPIC_0007_Wallets_Payments.xlsx
+++ b/EPIC_0007_Wallets_Payments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBA88A24-020A-491D-B279-CC674E5E755E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80908BEB-778A-4735-88BB-C6FC7998ED2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserDriverWebIntialilzer" sheetId="43" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="38">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -488,6 +488,18 @@
 70. Wait 3 seconds for the toast notification to hide.</t>
   </si>
   <si>
+    <t>34.Click Wallet,tap,,"mobile.customer.wallet.btn"
+35.Wait For Topup,wait_until_visible,,"mobile.customer.top_up.btn"
+36.Check Current Balance Displayed,element_present,,"mobile.customer.wallet.current_balance"
+37.Check Transaction History Displaye,element_present,,"mobile.customer.wallet.transaction_history"</t>
+  </si>
+  <si>
+    <t>TC_RG_02_Driver_App_Wallet_Verification</t>
+  </si>
+  <si>
+    <t>TC_RG_03_Customer_App_Wallet_Verification</t>
+  </si>
+  <si>
     <t>1. Load Driver App,switch_to,driver,
 2.Reload Driver App Completely,reload_app,driver,
 3. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
@@ -539,52 +551,224 @@
 49.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
 50.Click Success,tap,,"mobile.driver.top_up.succes_popup"
 51.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
-52.Click Back,tap,,"mobile.driver.back.btn"
-53.Drag Page Layout Upward,swipe,up,
-54.Click Back,tap,,"mobile.driver.back.btn"
-55.Reload Driver App Completely,reload_app,driver,
-56. Switch To Web Session,switch_to,web,
-57.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-58. Click Settings Menu,click,,"admin.setting.sidebar.menu"
-59. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-60. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-61.Wait For off,wait,2000,
-62. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
-63. Click Submit Button,click,,"web.global.action.submit"
-64. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-65. Switch To Driver Session,switch_to,driver,
-66. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-67. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-68. Click Agree,tap,,"mobile.driver.agree.btn"
-68. Click Get Started,tap,,"mobile.driver.get_started.btn"
-70. Click Next,tap,,"mobile.driver.next.btn"
-71. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-72. Click Close,tap,,"mobile.driver.cancel.btn"
-73. Enter Mobile Number,type,regression.approved_driver.phone ,"mobile.driver.edit_text.input"
-74. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-75. Click Continue,tap,,"mobile.driver.continue.btn"
-76. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-77. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-78. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-79.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
-80.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
-81.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"
-82.Load Super Admin,switch_to,web,
-83.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-84.Click Settings Menu,click,,"web.global.menu.settings"
-85.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-86.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-87.Wait For On,wait,2000,
-88.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
-89.Click Submit Button,click,,"web.global.action.submit"
-90.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-91.Wait For Toast To Hide,wait,3000,</t>
-  </si>
-  <si>
-    <t>34.Click Wallet,tap,,"mobile.customer.wallet.btn"
-35.Wait For Topup,wait_until_visible,,"mobile.customer.top_up.btn"
-36.Check Current Balance Displayed,element_present,,"mobile.customer.wallet.current_balance"
-37.Check Transaction History Displaye,element_present,,"mobile.customer.wallet.transaction_history"</t>
+52.Click Pay button,tap,,"mobile.driver.wallet_pay.btn"
+53.Click Benefical Search,tap,,"mobile.driver.wallet_pay.beneficial_search"
+54.Search Benfical Name,type,regression,"mobile.driver.wallet_pay.beneficial_search_Field"
+55.Enter Benfical Name,press_enter,,"mobile.driver.wallet_pay.beneficial_search_Field"
+56.Wait To Load,wait,3000
+57.Select Benefical,tap,,"mobile.driver.wallet_pay.beneficial_select"
+58.Enter Transfer Amout,type,100,"mobile.driver.wallet_pay.amount_field"
+59.Click Transfer Button,tap,,"mobile.driver.wallet_pay.transfer_btn"
+60.Wait For Transfer,wait,2000,
+61.Click Transfer Ok,tap,,"mobile.driver.wallet_pay.transfer_ok_btn"
+62.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
+63.Click Back,tap,,"mobile.driver.back.btn"
+64.Drag Page Layout Upward,swipe,up,
+65.Click Back,tap,,"mobile.driver.back.btn"
+66.Reload Driver App Completely,reload_app,driver,
+67. Switch To Web Session,switch_to,web,
+68.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+69. Click Settings Menu,click,,"admin.setting.sidebar.menu"
+70. Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+71. Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+72.Wait For off,wait,2000,
+73. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+74. Click Submit Button,click,,"web.global.action.submit"
+75. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+76. Switch To Driver Session,switch_to,driver,
+77. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+78. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+79. Click Agree,tap,,"mobile.driver.agree.btn"
+80. Click Get Started,tap,,"mobile.driver.get_started.btn"
+81. Click Next,tap,,"mobile.driver.next.btn"
+82. Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+83. Click Close,tap,,"mobile.driver.cancel.btn"
+84. Enter Mobile Number,type,regression.approved_driver.phone ,"mobile.driver.edit_text.input"
+85. Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+86. Click Continue,tap,,"mobile.driver.continue.btn"
+87. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+88. Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+89. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+90.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+91.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+92.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"
+93.Load Super Admin,switch_to,web,
+94.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+95.Click Settings Menu,click,,"web.global.menu.settings"
+96.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+97.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+98.Wait For On,wait,2000,
+99.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+100.Click Submit Button,click,,"web.global.action.submit"
+101.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+102.Wait For Toast To Hide,wait,3000,</t>
+  </si>
+  <si>
+    <t>1.Reload Driver App Completely,reload_app,driver,
+2.Load Super Admin,switch_to,web,
+3.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+4.Click Settings Menu,click,,"web.global.menu.settings"
+5.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+6.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+7.Wait For On,wait,2000,
+8.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+9.Click Submit Button,click,,"web.global.action.submit"
+10.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+11.Wait For Toast To Hide,wait,3000,
+12.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+13.Click drivers menu,click,,"admin.drivers.menu.icon"
+14.Click Add Driver menu,click,,"admin.drivers.add_menu.link"
+15.Verify Add Driver,verify,,"admin.drivers.add_page.header"
+16.Click Service Category Dropdown,click,,"admin.drivers.service_dropdown.select"
+17.Select Auto Ride Option,click,,"admin.drivers.service_dropdown.auto_ride"
+18.Click Driver Type Dropdown,click,,"admin.drivers.driver_type.dropdown"
+19.Select pilot Option,click,,"admin.drivers.driver_type.dropdown_pilot"
+20.Enter Driver Name, type, autodriver{randomAlpha} &gt;&gt; autoName, "admin.drivers.fullname.input"
+21.Enter Email, type, autodriver_{timestamp}@gmail.com&gt;&gt;autoEmail, "admin.drivers.email.input"
+22.Enter Contact Number, type, {randomPhone}&gt;&gt;autoPhone, "admin.drivers.phone.input"
+23.Click Whatspp, click, , "admin.drivers.whatsapp.checkbox"
+24.Enter Whatspp Number, type, {autoPhone}, "admin.drivers.whatsapp_phone.input"
+25.Upload Profile Image, uploadfile, "src/main/resources/test-data/autodriver.jpg", "admin.drivers.profile_image.file"
+26.Select Source,click,,"admin.drivers.source_dropdown.select"
+27.Select Instagram,click,,"admin.drivers.instagram_option.span"
+28.Select Male Gender, click, , "admin.drivers.male_gender.div"
+29.Click Vehicle Type Dropdown,click,,"admin.drivers.vehicle_dropdown.select"
+30. Select  Auto Option,click,,"admin.drivers.vehicle_option.pinkauto"
+31. Enter Model Year, type, 2013, "admin.drivers.modelyear.input"
+32. Enter Plate No, type, KL-01-AB-1234, "admin.drivers.plateno.input"
+33. Enter Model Name, type, petrol, "admin.drivers.modelname.input"
+34. Upload Vehicle Image, uploadfile, "src/main/resources/test-data/vehicle.jpg", "admin.drivers.vehicle_image.file"
+35. Enter Bank Name, type, HDFC Bank, "admin.drivers.bankname.input"
+36. Enter Bank Location, type, PARK STREET, "admin.drivers.banklocation.input"
+37. Enter Account Number, type, 50100123456789, "admin.drivers.accountno.input"
+38. Enter Account Holder Name, type,{autoName}, "admin.drivers.accountholder.input"
+39. Enter Payment Email Address, type, {autoEmail}, "admin.drivers.paymentemail.input"
+40. Enter IFSC Code, type, HDFC0001234, "admin.drivers.ifsc.input"
+41. Click Submit, click, , "web.global.action.submit"
+42. Verify Driver Added, verify,, "web.global.toast.success"
+43. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+44. Click drivers menu,click,,"admin.drivers.menu.icon"
+45. Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+46. Filter by Name,type,{autoName},"admin.drivers.name_filter.input"
+47. Scroll Grid, tab, 7, "admin.drivers.name_filter.input"
+48. Click Doc Icon,click,,"admin.drivers.docs.icon"
+49. Driver Required Documents,verify,,"admin.drivers.required_docs.header"
+50. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+51. Add Driving License,click,,"admin.drivers.docs.edit_icon"
+52. Upload Driving Iicense, uploadfile, "src/main/resources/test-data/license.jpg", "admin.drivers.profile_image.file"
+53. Enter Expiry Date,set_date,2026-12-12,"admin.drivers.doc_expiry.input"
+54. Click Submit, click, , "web.global.action.submit"
+55. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+56. Click Approve Driver,click,,"admin.drivers.docs.approval"
+57. Verify Updated Succesfully, verify, , "web.global.toast.updated"
+58. Click Dashboard,click,,"web.global.menu.dashboard"
+59. Click drivers menu,click,,"admin.drivers.menu.icon"
+60. Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+61. Approved Drivers List,verify,,"admin.drivers.approved_page.header"
+62. Filter Approved Driver,type,{autoName},"admin.drivers.name_filter.input"
+63.Wait For Load,wait,2000,
+64.Scroll Grid,tab,10,"admin.drivers.name_filter.input"
+65.Click Wallet,click,,"admin.drivers.wallet.btn"
+66.Click Manage Transaction,click,,"admin.drivers.wallet.manage_transaction.btn"
+67.Enter Wallet Amout,type,500,"admin.drivers.wallet.wallet_amount_input"
+68.Click Dropdown,click,,"admin.drivers.wallet.option_dropdown"
+69.Select Add Money Optin,click,,"admin.drivers.wallet.option_add_money"
+70.Click Submit Button,click,,"admin.drivers.wallet.submit.btn"
+71.Wait For Recharge,wait,2000,
+72.Load Driver App,switch_to,driver,
+73.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+74.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+75.Click Agree,tap,,"mobile.driver.agree.btn"
+76. Click Get Started,tap,,"mobile.driver.get_started.btn"
+77.Click Next,tap,,"mobile.driver.next.btn"
+78.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+79.Click Close,tap,,"mobile.driver.cancel.btn"
+80. Enter Mobile Number,type,{autoPhone},"mobile.driver.edit_text.input"
+81.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+82.Click Continue,tap,,"mobile.driver.continue.btn"
+83.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+84.Enter Account Holder,type,{autoName},"mobile.driver.bank_details.account_holder_name"
+85.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+86.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+87.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+88.Wait For Keyboard Minimises,hide_keyboard,,
+89.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
+90.Wait For Keyboard Minimises,hide_keyboard,,
+91.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+92.Force Driver Location To Perambur,set_location,13.121030;80.232578,
+93.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+94.Wait for Toast to Hide,wait,3000,,
+95.Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+96.Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+97.Click Agree,tap,,"mobile.driver.agree_continue.btn"
+98.Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+99. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+100. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+101.Wait For Hamburger Menu,wait,3000
+102.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+103.wait for Bank Details,wait_until_visible,"mobile.driver.bank_details.btn"
+104.Click Bank Details,tap,,"mobile.driver.bank_details.btn"
+105.Wait For Back,wait_until_visible,"mobile.driver.back.btn"
+106.Click Back,tap,,"mobile.driver.back.btn"
+107.wait for Wallet,wait_until_visible,"mobile.driver.wallet.btn"
+108.Click Wallet,tap,,"mobile.driver.wallet.btn"
+109.Wait For Topup,wait_until_visible,,"mobile.driver.top_up.btn"
+110.Check Current Balance Displayed,element_present,,"mobile.driver.wallet.current_balance"
+111.Check Transaction History Displaye,element_present,,"mobile.driver.wallet.transaction_history"
+112.Click Topup,tap,,"mobile.driver.top_up.btn"
+113.Wait For Topup Sum,wait_until_visible,,"mobile.driver.top_up.btn"
+114.Click Hundered,tap,,"mobile.driver.top_up_amount.hundred"
+115.Click Proceed,tap,,"mobile.driver.top_up.proceed"
+116.Wait For Contact No,wait_until_visible,,"mobile.driver.top_up.contact_no_box"
+117.Enter Driver Mobile,type,{autoPhone},"mobile.driver.top_up.contact_no_box"
+118.Wait For Payment Options,wait_until_visible,,"mobile.driver.top_up.payment_option"
+119.Wait For Net Banking,wait_until_visible,,"mobile.driver.top_up.net_banking"
+120.Click Net Banking,tap,,"mobile.driver.top_up.net_banking"
+121.Wait For Bob,wait_until_visible,,"mobile.driver.top_up.bob_bank"
+122.Click Bob,tap,,"mobile.driver.top_up.bob_bank"
+123.Wait For Success,wait_until_visible,,"mobile.driver.top_up.succes_popup"
+124.Click Success,tap,,"mobile.driver.top_up.succes_popup"
+125.Wait For Wallet  Back,wait_until_visible,,"mobile.driver.wallet.btn"
+126.Click Back,tap,,"mobile.driver.back.btn"
+127.Drag Page Layout Upward,swipe,up,
+128.Click Back,tap,,"mobile.driver.back.btn"
+129.Reload Driver App Completely,reload_app,driver,
+130.Switch To Web Session,switch_to,web,
+131.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+132.Click Settings Menu,click,,"admin.setting.sidebar.menu"
+133.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+134.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+135.Wait For off,wait,2000,
+136.Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+137.Click Submit Button,click,,"web.global.action.submit"
+138.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+139.Switch To Driver Session,switch_to,driver,
+140.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+141.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+142.Click Agree,tap,,"mobile.driver.agree.btn"
+143.Click Get Started,tap,,"mobile.driver.get_started.btn"
+144.Click Next,tap,,"mobile.driver.next.btn"
+145.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+146.Click Close,tap,,"mobile.driver.cancel.btn"
+147.Enter Mobile Number,type,{autoPhone} ,"mobile.driver.edit_text.input"
+148.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+149.Click Continue,tap,,"mobile.driver.continue.btn"
+150.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+151.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+152.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+153.Click Hamburger,tap_coordinate,75:209,COORDINATE_MODE
+154.Wait For Account,wait_until_visible,,"mobile.driver.account.heading"
+155.Check Wallet absent,element_absent,,"mobile.driver.wallet.btn"
+156.Load Super Admin,switch_to,web,
+157.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+158.Click Settings Menu,click,,"web.global.menu.settings"
+159.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+160.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+161.Wait For On,wait,2000,
+162.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+163.Click Submit Button,click,,"web.global.action.submit"
+164.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+165.Wait For Toast To Hide,wait,3000,</t>
   </si>
   <si>
     <t>1.Load User App,switch_to,user,
@@ -600,71 +784,84 @@
 11. Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
 12. Click Submit Button,click,,"web.global.action.submit"
 13. Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-14. Load User App,switch_to,user,
-15.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-16.Click Get Started,tap,,"mobile.customer.get_started.btn"
-17.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-18.Click Next,tap,,"mobile.customer.next.btn"
-19.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-20.Click Close,tap,,"mobile.customer.cancel.btn"
-21.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-22.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-23.Click Continue,tap,,"mobile.customer.continue.btn"
-24.Enter OTP,type,123456,"mobile.customer.otp_input"
-25.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-26.Click Finish,tap,,"mobile.customer.finish.btn"
-27.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-28. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
-29. Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
-30.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-31.wait for Wallet,wait_until_visible,"mobile.customer.wallet.btn"
-32.Check Wallet Present,element_present,,"mobile.customer.wallet.btn"
-33.Click Wallet,tap,,"mobile.customer.wallet.btn"
-34.Wait For Topup,wait_until_visible,,"mobile.customer.top_up.btn"
-35.Reload User App Completely,reload_app,user,
-36. Switch To Web Session,switch_to,web,
-37.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-38.Click Settings Menu,click,,"admin.setting.sidebar.menu"
-39.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-40.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-41.Wait For off,wait,2000,
-42. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
-43.Click Submit Button,click,,"web.global.action.submit"
-44.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-45.Load User App,switch_to,user,
-46.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
-47.Click Get Started,tap,,"mobile.customer.get_started.btn"
-48.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
-49.Click Next,tap,,"mobile.customer.next.btn"
-50.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
-51.Click Close,tap,,"mobile.customer.cancel.btn"
-52.Enter Mobile Number,type,regression.customer.phone,"mobile.customer.edit_text.input"
-53.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
-54.Click Continue,tap,,"mobile.customer.continue.btn"
-55.Enter OTP,type,123456,"mobile.customer.otp_input"
-56.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
-57.Click Finish,tap,,"mobile.customer.finish.btn"
-58.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
-59.Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
-60.Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
-61.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
-62.Check Wallet absent,element_absent,,"mobile.customer.wallet.btn"
-63.Load Super Admin,switch_to,web,
-64.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-65.Click Settings Menu,click,,"web.global.menu.settings"
-66.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
-67.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
-68.Wait For On,wait,2000,
-69.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
-70.Click Submit Button,click,,"web.global.action.submit"
-71.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
-72.Wait For Toast To Hide,wait,3000,</t>
-  </si>
-  <si>
-    <t>TC_RG_02_Driver_App_Wallet_Verification</t>
-  </si>
-  <si>
-    <t>TC_RG_03_Customer_App_Wallet_Verification</t>
+14. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+15.Click Customer Icon,click,,"admin.menu.customer_icon"
+16.Click Add Customers,click,,"admin.menu.add_customers"
+17.Wait For Customer Heading,wait_until_visible,,"admin.customer.add_heading"
+18.Enter Customer Name,type,customer{randomAlpha} &gt;&gt; customerName,"admin.customer.input_name"
+19.Enter Email,type,customer_{timestamp}@gmail.com&gt;&gt;customerEmail,"admin.customer.input_email"
+20.Enter Contact Number,type,{randomPhone}&gt;&gt;customerPhone,"admin.customer.input_phone"
+21.Enter Emergency Number,type,{randomPhone},"admin.customer.input_Emergency_phone"
+22.Open Gender,click,,"admin.customer.dropdown_gender"
+23.Select Male,click,,"admin.customer.select_gender_male"
+24.Upload Profile Image,uploadfile,"src/main/resources/test-data/customer.jpg","admin.customer.upload_profile_img"
+25.Click Submit,click,,"web.global.action.submit"
+26.Wait For Added Successfully,wait_until_visible,,"web.global.toast.info"
+27.Click Dashboard,click,,"web.global.menu.dashboard"
+28.Click Customer Icon,click,,"admin.menu.customer_icon"
+29.Click Verified Customers,click,,"admin.menu.verified_customers"
+30.Wait For Customer List Heading,wait_until_visible,,"admin.customer.verified_list_heading"
+31.Filter Customer Name List,type,{customerName},"admin.customer.filter_name"
+32.Wait For Load,wait,2000,
+33. Load User App,switch_to,user,
+34.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+35.Click Get Started,tap,,"mobile.customer.get_started.btn"
+36.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+37.Click Next,tap,,"mobile.customer.next.btn"
+38.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+39.Click Close,tap,,"mobile.customer.cancel.btn"
+40.Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+41.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+42.Click Continue,tap,,"mobile.customer.continue.btn"
+43.Enter OTP,type,123456,"mobile.customer.otp_input"
+44.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+45.Click Finish,tap,,"mobile.customer.finish.btn"
+46.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+47. Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+48.Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+49.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+50.wait for Wallet,wait_until_visible,"mobile.customer.wallet.btn"
+51.Check Wallet Present,element_present,,"mobile.customer.wallet.btn"
+52.Click Wallet,tap,,"mobile.customer.wallet.btn"
+53.Wait For Topup,wait_until_visible,,"mobile.customer.top_up.btn"
+54.Reload User App Completely,reload_app,user,
+55.Switch To Web Session,switch_to,web,
+56.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+57.Click Settings Menu,click,,"admin.setting.sidebar.menu"
+58.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+59.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+60.Wait For off,wait,2000,
+61. Select Wallet OFF Option,click,,"admin.setting.site_setting.walletdropdown_option_off"
+62.Click Submit Button,click,,"web.global.action.submit"
+63.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+64.Load User App,switch_to,user,
+65.Wait For Get Started,wait_until_visible,,"mobile.customer.get_started.btn"
+66.Click Get Started,tap,,"mobile.customer.get_started.btn"
+67.Click Allow Notification,tap,,"mobile.customer.permission_allow.btn"
+68.Click Next,tap,,"mobile.customer.next.btn"
+69.Click Mobile Number,tap,,"mobile.customer.mobile_number_field.btn"
+70.Click Close,tap,,"mobile.customer.cancel.btn"
+71.Enter Mobile Number,type,{customerPhone},"mobile.customer.edit_text.input"
+72.Wait for Continue,wait_until_visible,,"mobile.customer.continue.btn"
+73.Click Continue,tap,,"mobile.customer.continue.btn"
+74.Enter OTP,type,123456,"mobile.customer.otp_input"
+75.Wait for Finish,wait_until_visible,,"mobile.customer.finish.btn"
+76.Click Finish,tap,,"mobile.customer.finish.btn"
+77.Click Allow Location,tap,,"mobile.customer.location_allow.btn"
+78.Wait For Landing Page,wait_until_visible,,"mobile.customer.home_page.profile_icon"
+79.Click Profile_Menu,tap,,"mobile.customer.home_page.profile_icon"
+80.Wait For Profile,wait_until_visible,,"mobile.customer.account.heading"
+81.Check Wallet absent,element_absent,,"mobile.customer.wallet.btn"
+82.Load Super Admin,switch_to,web,
+83.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+84.Click Settings Menu,click,,"web.global.menu.settings"
+85.Click Site Settings Menu,click,,"admin.setting.site_setting.sidebar_menu"
+86.Click Wallet Status Dropdown,click,,"admin.setting.site_setting.wallet_dropdown"
+87.Wait For On,wait,2000,
+88.Select Wallet ON Option,click,,"admin.setting.site_setting.walletdropdown_option_on"
+89.Click Submit Button,click,,"web.global.action.submit"
+90.Verify Settings Updated Successfully,verify,,"web.global.toast.updated"
+91.Wait For Toast To Hide,wait,3000,</t>
   </si>
 </sst>
 </file>
@@ -1119,8 +1316,8 @@
     <col min="6" max="6" width="45.77734375" customWidth="1"/>
     <col min="7" max="7" width="71.44140625" customWidth="1"/>
     <col min="8" max="8" width="40.44140625" customWidth="1"/>
-    <col min="9" max="9" width="61.88671875" customWidth="1"/>
-    <col min="10" max="10" width="32.88671875" customWidth="1"/>
+    <col min="9" max="9" width="25.88671875" customWidth="1"/>
+    <col min="10" max="10" width="66.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1166,7 +1363,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>25</v>
@@ -1175,7 +1372,7 @@
         <v>26</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -1183,7 +1380,9 @@
       <c r="I2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="2"/>
+      <c r="J2" s="2" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
@@ -1264,7 +1463,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>29</v>
@@ -1273,7 +1472,7 @@
         <v>31</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -1282,7 +1481,7 @@
         <v>30</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>